<commit_message>
chore: atualiza histórico de ordens 2026-08-21
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,6 +1059,615 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>26.08</v>
+      </c>
+      <c r="D31" t="n">
+        <v>28</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>12.84</v>
+      </c>
+      <c r="D32" t="n">
+        <v>31</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="D33" t="n">
+        <v>30</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="D34" t="n">
+        <v>16</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D35" t="n">
+        <v>12</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>168.33</v>
+      </c>
+      <c r="D36" t="n">
+        <v>26</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>51.85</v>
+      </c>
+      <c r="D37" t="n">
+        <v>45</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="D38" t="n">
+        <v>61</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="D39" t="n">
+        <v>10</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="D40" t="n">
+        <v>22</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="D41" t="n">
+        <v>49</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="D42" t="n">
+        <v>20</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="D44" t="n">
+        <v>26</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>21.17</v>
+      </c>
+      <c r="D45" t="n">
+        <v>27</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="D46" t="n">
+        <v>22</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="D47" t="n">
+        <v>20</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="D48" t="n">
+        <v>25</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="D49" t="n">
+        <v>30</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>23</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="D51" t="n">
+        <v>20</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>62.85</v>
+      </c>
+      <c r="D52" t="n">
+        <v>8</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>46.57</v>
+      </c>
+      <c r="D53" t="n">
+        <v>16</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="D54" t="n">
+        <v>63</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>34.25</v>
+      </c>
+      <c r="D55" t="n">
+        <v>35</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="D56" t="n">
+        <v>31</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>44.97</v>
+      </c>
+      <c r="D57" t="n">
+        <v>11</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="D58" t="n">
+        <v>11</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>34.61</v>
+      </c>
+      <c r="D59" t="n">
+        <v>48</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-24
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1060,7 +1060,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B50" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B51" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B52" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B53" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B54" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B55" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B56" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B57" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B58" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="B59" t="inlineStr">
@@ -1663,6 +1663,615 @@
         <v>48</v>
       </c>
       <c r="E59" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>26.01</v>
+      </c>
+      <c r="D60" t="n">
+        <v>28</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D61" t="n">
+        <v>31</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D62" t="n">
+        <v>30</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="D63" t="n">
+        <v>16</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D64" t="n">
+        <v>12</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>169.01</v>
+      </c>
+      <c r="D65" t="n">
+        <v>26</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="D66" t="n">
+        <v>45</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="D67" t="n">
+        <v>61</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="D68" t="n">
+        <v>10</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="D69" t="n">
+        <v>22</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D70" t="n">
+        <v>49</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>20</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="D72" t="n">
+        <v>9</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D73" t="n">
+        <v>26</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>21.42</v>
+      </c>
+      <c r="D74" t="n">
+        <v>27</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D75" t="n">
+        <v>22</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="D76" t="n">
+        <v>20</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="D77" t="n">
+        <v>25</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="D78" t="n">
+        <v>30</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>42.11</v>
+      </c>
+      <c r="D79" t="n">
+        <v>23</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="D80" t="n">
+        <v>20</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>61.62</v>
+      </c>
+      <c r="D81" t="n">
+        <v>8</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>47.59</v>
+      </c>
+      <c r="D82" t="n">
+        <v>16</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>18.32</v>
+      </c>
+      <c r="D83" t="n">
+        <v>63</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>34.52</v>
+      </c>
+      <c r="D84" t="n">
+        <v>35</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>102.64</v>
+      </c>
+      <c r="D85" t="n">
+        <v>31</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="D86" t="n">
+        <v>11</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="D87" t="n">
+        <v>11</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>33.86</v>
+      </c>
+      <c r="D88" t="n">
+        <v>48</v>
+      </c>
+      <c r="E88" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-25
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1669,7 +1669,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B60" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B61" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B62" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B63" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B64" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B65" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B66" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B67" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B68" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B69" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B70" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B71" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B72" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B73" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B74" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B75" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B76" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B77" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B78" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B79" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B80" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B81" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B82" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B83" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B84" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B85" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B86" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B87" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>46258</v>
       </c>
       <c r="B88" t="inlineStr">
@@ -2272,6 +2272,615 @@
         <v>48</v>
       </c>
       <c r="E88" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>26.56</v>
+      </c>
+      <c r="D89" t="n">
+        <v>28</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>13.24</v>
+      </c>
+      <c r="D90" t="n">
+        <v>31</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="D91" t="n">
+        <v>30</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="D92" t="n">
+        <v>16</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="D93" t="n">
+        <v>12</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>171.88</v>
+      </c>
+      <c r="D94" t="n">
+        <v>26</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="D95" t="n">
+        <v>45</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="D96" t="n">
+        <v>61</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="D97" t="n">
+        <v>10</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="D98" t="n">
+        <v>22</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>19.14</v>
+      </c>
+      <c r="D99" t="n">
+        <v>49</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>26.69</v>
+      </c>
+      <c r="D100" t="n">
+        <v>20</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="D101" t="n">
+        <v>9</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="D102" t="n">
+        <v>26</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="D103" t="n">
+        <v>27</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="D104" t="n">
+        <v>22</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="D105" t="n">
+        <v>20</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="D106" t="n">
+        <v>25</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="D107" t="n">
+        <v>30</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>41.35</v>
+      </c>
+      <c r="D108" t="n">
+        <v>23</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="D109" t="n">
+        <v>20</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>60.88</v>
+      </c>
+      <c r="D110" t="n">
+        <v>8</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="D111" t="n">
+        <v>16</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>19.59</v>
+      </c>
+      <c r="D112" t="n">
+        <v>63</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>36.07</v>
+      </c>
+      <c r="D113" t="n">
+        <v>35</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>105.24</v>
+      </c>
+      <c r="D114" t="n">
+        <v>31</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>46.34</v>
+      </c>
+      <c r="D115" t="n">
+        <v>11</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="D116" t="n">
+        <v>11</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>34.09</v>
+      </c>
+      <c r="D117" t="n">
+        <v>48</v>
+      </c>
+      <c r="E117" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-27
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2278,7 +2278,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B89" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B90" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B91" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B92" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B93" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B94" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B95" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B96" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B97" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B98" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B99" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B100" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B101" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B102" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B103" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B104" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B105" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B106" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B107" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B108" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B109" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B110" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B111" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B112" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B113" t="inlineStr">
@@ -2803,7 +2803,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B114" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B115" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B116" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="B117" t="inlineStr">
@@ -2881,6 +2881,615 @@
         <v>48</v>
       </c>
       <c r="E117" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>26.43000030517578</v>
+      </c>
+      <c r="D118" t="n">
+        <v>28</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>13.60000038146973</v>
+      </c>
+      <c r="D119" t="n">
+        <v>31</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>19.52000045776367</v>
+      </c>
+      <c r="D120" t="n">
+        <v>30</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>4.099999904632568</v>
+      </c>
+      <c r="D121" t="n">
+        <v>16</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>0.3600000143051147</v>
+      </c>
+      <c r="D122" t="n">
+        <v>12</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>171.8200073242188</v>
+      </c>
+      <c r="D123" t="n">
+        <v>26</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>54.06999969482422</v>
+      </c>
+      <c r="D124" t="n">
+        <v>45</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>3.519999980926514</v>
+      </c>
+      <c r="D125" t="n">
+        <v>61</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>5.989999771118164</v>
+      </c>
+      <c r="D126" t="n">
+        <v>10</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>5.269999980926514</v>
+      </c>
+      <c r="D127" t="n">
+        <v>22</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>19.20999908447266</v>
+      </c>
+      <c r="D128" t="n">
+        <v>49</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>26.3799991607666</v>
+      </c>
+      <c r="D129" t="n">
+        <v>20</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>11.55000019073486</v>
+      </c>
+      <c r="D130" t="n">
+        <v>9</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>4.599999904632568</v>
+      </c>
+      <c r="D131" t="n">
+        <v>26</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>22.01000022888184</v>
+      </c>
+      <c r="D132" t="n">
+        <v>27</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>10.39999961853027</v>
+      </c>
+      <c r="D133" t="n">
+        <v>22</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>4.710000038146973</v>
+      </c>
+      <c r="D134" t="n">
+        <v>20</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>7.190000057220459</v>
+      </c>
+      <c r="D135" t="n">
+        <v>25</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>5.510000228881836</v>
+      </c>
+      <c r="D136" t="n">
+        <v>30</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>41.45000076293945</v>
+      </c>
+      <c r="D137" t="n">
+        <v>23</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>4.409999847412109</v>
+      </c>
+      <c r="D138" t="n">
+        <v>20</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>60.7599983215332</v>
+      </c>
+      <c r="D139" t="n">
+        <v>8</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>48.54000091552734</v>
+      </c>
+      <c r="D140" t="n">
+        <v>16</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>19.30999946594238</v>
+      </c>
+      <c r="D141" t="n">
+        <v>63</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>35.29999923706055</v>
+      </c>
+      <c r="D142" t="n">
+        <v>35</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>104.8000030517578</v>
+      </c>
+      <c r="D143" t="n">
+        <v>31</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>46.15000152587891</v>
+      </c>
+      <c r="D144" t="n">
+        <v>11</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>7.130000114440918</v>
+      </c>
+      <c r="D145" t="n">
+        <v>11</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>33.61000061035156</v>
+      </c>
+      <c r="D146" t="n">
+        <v>48</v>
+      </c>
+      <c r="E146" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-28
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3496,7 +3496,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B147" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B148" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B149" t="inlineStr">
@@ -3559,7 +3559,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B150" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B151" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B152" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B153" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B154" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B155" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B156" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B157" t="inlineStr">
@@ -3727,7 +3727,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B158" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B159" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B160" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B161" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B162" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B163" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B164" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B165" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B166" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B167" t="inlineStr">
@@ -3937,7 +3937,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B168" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B169" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B170" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B171" t="inlineStr">
@@ -4021,7 +4021,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B172" t="inlineStr">
@@ -4042,7 +4042,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B173" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B174" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="B175" t="inlineStr">
@@ -4099,6 +4099,615 @@
         <v>48</v>
       </c>
       <c r="E175" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="D176" t="n">
+        <v>28</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>14.32</v>
+      </c>
+      <c r="D177" t="n">
+        <v>31</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="D178" t="n">
+        <v>30</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="D179" t="n">
+        <v>16</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D180" t="n">
+        <v>12</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>172.4</v>
+      </c>
+      <c r="D181" t="n">
+        <v>26</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>53.74</v>
+      </c>
+      <c r="D182" t="n">
+        <v>45</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="D183" t="n">
+        <v>61</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="D184" t="n">
+        <v>10</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="D185" t="n">
+        <v>22</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>19.31</v>
+      </c>
+      <c r="D186" t="n">
+        <v>49</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>26.15</v>
+      </c>
+      <c r="D187" t="n">
+        <v>20</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>11.77</v>
+      </c>
+      <c r="D188" t="n">
+        <v>9</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="D189" t="n">
+        <v>26</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="D190" t="n">
+        <v>27</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="D191" t="n">
+        <v>22</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="D192" t="n">
+        <v>20</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="D193" t="n">
+        <v>25</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="D194" t="n">
+        <v>30</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="D195" t="n">
+        <v>23</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D196" t="n">
+        <v>20</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="D197" t="n">
+        <v>8</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="D198" t="n">
+        <v>16</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D199" t="n">
+        <v>63</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>35.31</v>
+      </c>
+      <c r="D200" t="n">
+        <v>35</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>105.17</v>
+      </c>
+      <c r="D201" t="n">
+        <v>31</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="D202" t="n">
+        <v>11</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="D203" t="n">
+        <v>11</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>33.35</v>
+      </c>
+      <c r="D204" t="n">
+        <v>48</v>
+      </c>
+      <c r="E204" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
projeto_hilo.py: idempotente por dia (substitui em vez de só concatenar) -- evita duplicar linha se o workflow rodar 2x no mesmo dia; limpa as duplicatas já existentes (achado em 27/08 e histórico anterior)
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -16,11 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,10 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E204"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2896,7 +2893,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>26.43000030517578</v>
+        <v>26.43</v>
       </c>
       <c r="D118" t="n">
         <v>28</v>
@@ -2917,7 +2914,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>13.60000038146973</v>
+        <v>13.6</v>
       </c>
       <c r="D119" t="n">
         <v>31</v>
@@ -2938,7 +2935,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>19.52000045776367</v>
+        <v>19.52</v>
       </c>
       <c r="D120" t="n">
         <v>30</v>
@@ -2959,7 +2956,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4.099999904632568</v>
+        <v>4.1</v>
       </c>
       <c r="D121" t="n">
         <v>16</v>
@@ -2980,7 +2977,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>0.3600000143051147</v>
+        <v>0.36</v>
       </c>
       <c r="D122" t="n">
         <v>12</v>
@@ -3001,7 +2998,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>171.8200073242188</v>
+        <v>171.82</v>
       </c>
       <c r="D123" t="n">
         <v>26</v>
@@ -3022,7 +3019,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>54.06999969482422</v>
+        <v>54.07</v>
       </c>
       <c r="D124" t="n">
         <v>45</v>
@@ -3043,7 +3040,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>3.519999980926514</v>
+        <v>3.52</v>
       </c>
       <c r="D125" t="n">
         <v>61</v>
@@ -3064,7 +3061,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>5.989999771118164</v>
+        <v>5.99</v>
       </c>
       <c r="D126" t="n">
         <v>10</v>
@@ -3085,7 +3082,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>5.269999980926514</v>
+        <v>5.27</v>
       </c>
       <c r="D127" t="n">
         <v>22</v>
@@ -3106,7 +3103,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>19.20999908447266</v>
+        <v>19.21</v>
       </c>
       <c r="D128" t="n">
         <v>49</v>
@@ -3127,7 +3124,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>26.3799991607666</v>
+        <v>26.38</v>
       </c>
       <c r="D129" t="n">
         <v>20</v>
@@ -3148,7 +3145,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>11.55000019073486</v>
+        <v>11.55</v>
       </c>
       <c r="D130" t="n">
         <v>9</v>
@@ -3169,7 +3166,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>4.599999904632568</v>
+        <v>4.6</v>
       </c>
       <c r="D131" t="n">
         <v>26</v>
@@ -3190,7 +3187,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>22.01000022888184</v>
+        <v>22.01</v>
       </c>
       <c r="D132" t="n">
         <v>27</v>
@@ -3211,7 +3208,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>10.39999961853027</v>
+        <v>10.4</v>
       </c>
       <c r="D133" t="n">
         <v>22</v>
@@ -3232,7 +3229,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>4.710000038146973</v>
+        <v>4.71</v>
       </c>
       <c r="D134" t="n">
         <v>20</v>
@@ -3253,7 +3250,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>7.190000057220459</v>
+        <v>7.19</v>
       </c>
       <c r="D135" t="n">
         <v>25</v>
@@ -3274,7 +3271,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>5.510000228881836</v>
+        <v>5.51</v>
       </c>
       <c r="D136" t="n">
         <v>30</v>
@@ -3295,7 +3292,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>41.45000076293945</v>
+        <v>41.45</v>
       </c>
       <c r="D137" t="n">
         <v>23</v>
@@ -3316,7 +3313,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>4.409999847412109</v>
+        <v>4.41</v>
       </c>
       <c r="D138" t="n">
         <v>20</v>
@@ -3337,7 +3334,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>60.7599983215332</v>
+        <v>60.76</v>
       </c>
       <c r="D139" t="n">
         <v>8</v>
@@ -3358,7 +3355,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>48.54000091552734</v>
+        <v>48.54</v>
       </c>
       <c r="D140" t="n">
         <v>16</v>
@@ -3379,7 +3376,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>19.30999946594238</v>
+        <v>19.31</v>
       </c>
       <c r="D141" t="n">
         <v>63</v>
@@ -3400,7 +3397,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>35.29999923706055</v>
+        <v>35.3</v>
       </c>
       <c r="D142" t="n">
         <v>35</v>
@@ -3421,7 +3418,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>104.8000030517578</v>
+        <v>104.8</v>
       </c>
       <c r="D143" t="n">
         <v>31</v>
@@ -3442,7 +3439,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>46.15000152587891</v>
+        <v>46.15</v>
       </c>
       <c r="D144" t="n">
         <v>11</v>
@@ -3463,7 +3460,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>7.130000114440918</v>
+        <v>7.13</v>
       </c>
       <c r="D145" t="n">
         <v>11</v>
@@ -3484,7 +3481,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>33.61000061035156</v>
+        <v>33.61</v>
       </c>
       <c r="D146" t="n">
         <v>48</v>
@@ -3497,7 +3494,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -3505,7 +3502,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>26.43</v>
+        <v>26.21</v>
       </c>
       <c r="D147" t="n">
         <v>28</v>
@@ -3518,7 +3515,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -3526,7 +3523,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>13.6</v>
+        <v>14.32</v>
       </c>
       <c r="D148" t="n">
         <v>31</v>
@@ -3539,7 +3536,7 @@
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -3547,7 +3544,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>19.52</v>
+        <v>19.97</v>
       </c>
       <c r="D149" t="n">
         <v>30</v>
@@ -3560,7 +3557,7 @@
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -3568,7 +3565,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>4.1</v>
+        <v>3.97</v>
       </c>
       <c r="D150" t="n">
         <v>16</v>
@@ -3581,7 +3578,7 @@
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -3589,7 +3586,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="D151" t="n">
         <v>12</v>
@@ -3602,7 +3599,7 @@
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -3610,7 +3607,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>171.82</v>
+        <v>172.4</v>
       </c>
       <c r="D152" t="n">
         <v>26</v>
@@ -3623,7 +3620,7 @@
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -3631,7 +3628,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>54.07</v>
+        <v>53.74</v>
       </c>
       <c r="D153" t="n">
         <v>45</v>
@@ -3644,7 +3641,7 @@
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -3652,7 +3649,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3.52</v>
+        <v>4.22</v>
       </c>
       <c r="D154" t="n">
         <v>61</v>
@@ -3665,7 +3662,7 @@
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -3673,7 +3670,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>5.99</v>
+        <v>6.01</v>
       </c>
       <c r="D155" t="n">
         <v>10</v>
@@ -3686,7 +3683,7 @@
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -3694,7 +3691,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>5.27</v>
+        <v>5.37</v>
       </c>
       <c r="D156" t="n">
         <v>22</v>
@@ -3707,7 +3704,7 @@
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -3715,7 +3712,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>19.21</v>
+        <v>19.31</v>
       </c>
       <c r="D157" t="n">
         <v>49</v>
@@ -3728,7 +3725,7 @@
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -3736,7 +3733,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>26.38</v>
+        <v>26.15</v>
       </c>
       <c r="D158" t="n">
         <v>20</v>
@@ -3749,7 +3746,7 @@
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -3757,7 +3754,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>11.55</v>
+        <v>11.77</v>
       </c>
       <c r="D159" t="n">
         <v>9</v>
@@ -3770,7 +3767,7 @@
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -3778,7 +3775,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>4.6</v>
+        <v>4.76</v>
       </c>
       <c r="D160" t="n">
         <v>26</v>
@@ -3791,7 +3788,7 @@
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -3799,7 +3796,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>22.01</v>
+        <v>21.25</v>
       </c>
       <c r="D161" t="n">
         <v>27</v>
@@ -3812,7 +3809,7 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -3820,7 +3817,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>10.4</v>
+        <v>10.36</v>
       </c>
       <c r="D162" t="n">
         <v>22</v>
@@ -3833,7 +3830,7 @@
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -3841,7 +3838,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>4.71</v>
+        <v>4.84</v>
       </c>
       <c r="D163" t="n">
         <v>20</v>
@@ -3854,7 +3851,7 @@
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -3862,7 +3859,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>7.19</v>
+        <v>7.21</v>
       </c>
       <c r="D164" t="n">
         <v>25</v>
@@ -3875,7 +3872,7 @@
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -3883,7 +3880,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>5.51</v>
+        <v>5.47</v>
       </c>
       <c r="D165" t="n">
         <v>30</v>
@@ -3896,7 +3893,7 @@
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -3904,7 +3901,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>41.45</v>
+        <v>42.7</v>
       </c>
       <c r="D166" t="n">
         <v>23</v>
@@ -3917,7 +3914,7 @@
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -3925,7 +3922,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4.41</v>
+        <v>4.5</v>
       </c>
       <c r="D167" t="n">
         <v>20</v>
@@ -3938,7 +3935,7 @@
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -3946,7 +3943,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>60.76</v>
+        <v>61.09</v>
       </c>
       <c r="D168" t="n">
         <v>8</v>
@@ -3959,7 +3956,7 @@
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -3967,7 +3964,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>48.54</v>
+        <v>48.34</v>
       </c>
       <c r="D169" t="n">
         <v>16</v>
@@ -3980,7 +3977,7 @@
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -3988,7 +3985,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>19.31</v>
+        <v>19.4</v>
       </c>
       <c r="D170" t="n">
         <v>63</v>
@@ -4001,7 +3998,7 @@
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -4009,7 +4006,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>35.3</v>
+        <v>35.31</v>
       </c>
       <c r="D171" t="n">
         <v>35</v>
@@ -4022,7 +4019,7 @@
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -4030,7 +4027,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>104.8</v>
+        <v>105.17</v>
       </c>
       <c r="D172" t="n">
         <v>31</v>
@@ -4043,7 +4040,7 @@
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -4051,7 +4048,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>46.15</v>
+        <v>46.4</v>
       </c>
       <c r="D173" t="n">
         <v>11</v>
@@ -4064,7 +4061,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -4072,7 +4069,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>7.13</v>
+        <v>7.17</v>
       </c>
       <c r="D174" t="n">
         <v>11</v>
@@ -4085,7 +4082,7 @@
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -4093,621 +4090,12 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>33.61</v>
+        <v>33.35</v>
       </c>
       <c r="D175" t="n">
         <v>48</v>
       </c>
       <c r="E175" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>ALOS3</t>
-        </is>
-      </c>
-      <c r="C176" t="n">
-        <v>26.21</v>
-      </c>
-      <c r="D176" t="n">
-        <v>28</v>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>ALPA4</t>
-        </is>
-      </c>
-      <c r="C177" t="n">
-        <v>14.32</v>
-      </c>
-      <c r="D177" t="n">
-        <v>31</v>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>BBAS3</t>
-        </is>
-      </c>
-      <c r="C178" t="n">
-        <v>19.97</v>
-      </c>
-      <c r="D178" t="n">
-        <v>30</v>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>BEEF3</t>
-        </is>
-      </c>
-      <c r="C179" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="D179" t="n">
-        <v>16</v>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>BHIA3</t>
-        </is>
-      </c>
-      <c r="C180" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="D180" t="n">
-        <v>12</v>
-      </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>BOVA11</t>
-        </is>
-      </c>
-      <c r="C181" t="n">
-        <v>172.4</v>
-      </c>
-      <c r="D181" t="n">
-        <v>26</v>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>BPAC11</t>
-        </is>
-      </c>
-      <c r="C182" t="n">
-        <v>53.74</v>
-      </c>
-      <c r="D182" t="n">
-        <v>45</v>
-      </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>BRKM5</t>
-        </is>
-      </c>
-      <c r="C183" t="n">
-        <v>4.22</v>
-      </c>
-      <c r="D183" t="n">
-        <v>61</v>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>CMIN3</t>
-        </is>
-      </c>
-      <c r="C184" t="n">
-        <v>6.01</v>
-      </c>
-      <c r="D184" t="n">
-        <v>10</v>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>CSNA3</t>
-        </is>
-      </c>
-      <c r="C185" t="n">
-        <v>5.37</v>
-      </c>
-      <c r="D185" t="n">
-        <v>22</v>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>CXSE3</t>
-        </is>
-      </c>
-      <c r="C186" t="n">
-        <v>19.31</v>
-      </c>
-      <c r="D186" t="n">
-        <v>49</v>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>ENEV3</t>
-        </is>
-      </c>
-      <c r="C187" t="n">
-        <v>26.15</v>
-      </c>
-      <c r="D187" t="n">
-        <v>20</v>
-      </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>EZTC3</t>
-        </is>
-      </c>
-      <c r="C188" t="n">
-        <v>11.77</v>
-      </c>
-      <c r="D188" t="n">
-        <v>9</v>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>GMAT3</t>
-        </is>
-      </c>
-      <c r="C189" t="n">
-        <v>4.76</v>
-      </c>
-      <c r="D189" t="n">
-        <v>26</v>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>HYPE3</t>
-        </is>
-      </c>
-      <c r="C190" t="n">
-        <v>21.25</v>
-      </c>
-      <c r="D190" t="n">
-        <v>27</v>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>JHSF3</t>
-        </is>
-      </c>
-      <c r="C191" t="n">
-        <v>10.36</v>
-      </c>
-      <c r="D191" t="n">
-        <v>22</v>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>MGLU3</t>
-        </is>
-      </c>
-      <c r="C192" t="n">
-        <v>4.84</v>
-      </c>
-      <c r="D192" t="n">
-        <v>20</v>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>MOVI3</t>
-        </is>
-      </c>
-      <c r="C193" t="n">
-        <v>7.21</v>
-      </c>
-      <c r="D193" t="n">
-        <v>25</v>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>MRVE3</t>
-        </is>
-      </c>
-      <c r="C194" t="n">
-        <v>5.47</v>
-      </c>
-      <c r="D194" t="n">
-        <v>30</v>
-      </c>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>PETR4</t>
-        </is>
-      </c>
-      <c r="C195" t="n">
-        <v>42.7</v>
-      </c>
-      <c r="D195" t="n">
-        <v>23</v>
-      </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>POMO4</t>
-        </is>
-      </c>
-      <c r="C196" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D196" t="n">
-        <v>20</v>
-      </c>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>PRIO3</t>
-        </is>
-      </c>
-      <c r="C197" t="n">
-        <v>61.09</v>
-      </c>
-      <c r="D197" t="n">
-        <v>8</v>
-      </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>PSSA3</t>
-        </is>
-      </c>
-      <c r="C198" t="n">
-        <v>48.34</v>
-      </c>
-      <c r="D198" t="n">
-        <v>16</v>
-      </c>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>RADL3</t>
-        </is>
-      </c>
-      <c r="C199" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="D199" t="n">
-        <v>63</v>
-      </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>RDOR3</t>
-        </is>
-      </c>
-      <c r="C200" t="n">
-        <v>35.31</v>
-      </c>
-      <c r="D200" t="n">
-        <v>35</v>
-      </c>
-      <c r="E200" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>SMAL11</t>
-        </is>
-      </c>
-      <c r="C201" t="n">
-        <v>105.17</v>
-      </c>
-      <c r="D201" t="n">
-        <v>31</v>
-      </c>
-      <c r="E201" t="inlineStr">
-        <is>
-          <t>Venda</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>SUZB3</t>
-        </is>
-      </c>
-      <c r="C202" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="D202" t="n">
-        <v>11</v>
-      </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>USIM5</t>
-        </is>
-      </c>
-      <c r="C203" t="n">
-        <v>7.17</v>
-      </c>
-      <c r="D203" t="n">
-        <v>11</v>
-      </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>Compra</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="2" t="n">
-        <v>46262</v>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>VBBR3</t>
-        </is>
-      </c>
-      <c r="C204" t="n">
-        <v>33.35</v>
-      </c>
-      <c r="D204" t="n">
-        <v>48</v>
-      </c>
-      <c r="E204" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-29
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4101,6 +4104,557 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr"/>
+      <c r="D176" t="n">
+        <v>28</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="n">
+        <v>31</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr"/>
+      <c r="D178" t="n">
+        <v>30</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr"/>
+      <c r="D179" t="n">
+        <v>16</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr"/>
+      <c r="D180" t="n">
+        <v>12</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr"/>
+      <c r="D181" t="n">
+        <v>26</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr"/>
+      <c r="D182" t="n">
+        <v>45</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="n">
+        <v>61</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr"/>
+      <c r="D184" t="n">
+        <v>10</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr"/>
+      <c r="D185" t="n">
+        <v>22</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" t="n">
+        <v>49</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr"/>
+      <c r="D187" t="n">
+        <v>20</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr"/>
+      <c r="D188" t="n">
+        <v>9</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr"/>
+      <c r="D189" t="n">
+        <v>26</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr"/>
+      <c r="D190" t="n">
+        <v>27</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr"/>
+      <c r="D191" t="n">
+        <v>22</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr"/>
+      <c r="D192" t="n">
+        <v>20</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr"/>
+      <c r="D193" t="n">
+        <v>25</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr"/>
+      <c r="D194" t="n">
+        <v>30</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr"/>
+      <c r="D195" t="n">
+        <v>23</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr"/>
+      <c r="D196" t="n">
+        <v>20</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr"/>
+      <c r="D197" t="n">
+        <v>8</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr"/>
+      <c r="D198" t="n">
+        <v>16</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr"/>
+      <c r="D199" t="n">
+        <v>63</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr"/>
+      <c r="D200" t="n">
+        <v>35</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr"/>
+      <c r="D201" t="n">
+        <v>31</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr"/>
+      <c r="D202" t="n">
+        <v>11</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr"/>
+      <c r="D203" t="n">
+        <v>11</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr"/>
+      <c r="D204" t="n">
+        <v>48</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-08-31
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E204"/>
+  <dimension ref="A1:E233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4105,7 +4105,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B176" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B177" t="inlineStr">
@@ -4143,7 +4143,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B178" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B179" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B180" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B181" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B182" t="inlineStr">
@@ -4238,7 +4238,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B183" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B184" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B185" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B186" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B187" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B188" t="inlineStr">
@@ -4352,7 +4352,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B189" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B190" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B191" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B192" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B193" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B194" t="inlineStr">
@@ -4466,7 +4466,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B195" t="inlineStr">
@@ -4485,7 +4485,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B196" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B197" t="inlineStr">
@@ -4523,7 +4523,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B198" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B199" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B200" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B201" t="inlineStr">
@@ -4599,7 +4599,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B202" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B203" t="inlineStr">
@@ -4637,7 +4637,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="B204" t="inlineStr">
@@ -4650,6 +4650,615 @@
         <v>48</v>
       </c>
       <c r="E204" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>26.69</v>
+      </c>
+      <c r="D205" t="n">
+        <v>28</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="D206" t="n">
+        <v>31</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>20.74</v>
+      </c>
+      <c r="D207" t="n">
+        <v>30</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="D208" t="n">
+        <v>16</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D209" t="n">
+        <v>12</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>174.78</v>
+      </c>
+      <c r="D210" t="n">
+        <v>26</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>54.71</v>
+      </c>
+      <c r="D211" t="n">
+        <v>45</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="D212" t="n">
+        <v>61</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="D213" t="n">
+        <v>10</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="D214" t="n">
+        <v>22</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>19.34</v>
+      </c>
+      <c r="D215" t="n">
+        <v>49</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="D216" t="n">
+        <v>20</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="D217" t="n">
+        <v>9</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="D218" t="n">
+        <v>26</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D219" t="n">
+        <v>27</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="D220" t="n">
+        <v>22</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="D221" t="n">
+        <v>20</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="D222" t="n">
+        <v>25</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="D223" t="n">
+        <v>30</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>45.02</v>
+      </c>
+      <c r="D224" t="n">
+        <v>23</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D225" t="n">
+        <v>20</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>62.68</v>
+      </c>
+      <c r="D226" t="n">
+        <v>8</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>49.08</v>
+      </c>
+      <c r="D227" t="n">
+        <v>16</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D228" t="n">
+        <v>63</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>35.18</v>
+      </c>
+      <c r="D229" t="n">
+        <v>35</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>106.13</v>
+      </c>
+      <c r="D230" t="n">
+        <v>31</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="D231" t="n">
+        <v>11</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="D232" t="n">
+        <v>11</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>34.42</v>
+      </c>
+      <c r="D233" t="n">
+        <v>48</v>
+      </c>
+      <c r="E233" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-01
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E233"/>
+  <dimension ref="A1:E262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4656,7 +4656,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B205" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B206" t="inlineStr">
@@ -4698,7 +4698,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B207" t="inlineStr">
@@ -4719,7 +4719,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B208" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B209" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B210" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B211" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B212" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B213" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B214" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B215" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B216" t="inlineStr">
@@ -4908,7 +4908,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B217" t="inlineStr">
@@ -4929,7 +4929,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B218" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B219" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B220" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B221" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B222" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B223" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B224" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B225" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B226" t="inlineStr">
@@ -5118,7 +5118,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B227" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B228" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B229" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B230" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B231" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B232" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B233" t="inlineStr">
@@ -5259,6 +5259,615 @@
         <v>48</v>
       </c>
       <c r="E233" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>26.69000053405762</v>
+      </c>
+      <c r="D234" t="n">
+        <v>28</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>14.98999977111816</v>
+      </c>
+      <c r="D235" t="n">
+        <v>31</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>20.73999977111816</v>
+      </c>
+      <c r="D236" t="n">
+        <v>30</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>3.819999933242798</v>
+      </c>
+      <c r="D237" t="n">
+        <v>16</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>0.6600000262260437</v>
+      </c>
+      <c r="D238" t="n">
+        <v>12</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>174.7799987792969</v>
+      </c>
+      <c r="D239" t="n">
+        <v>26</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>54.70999908447266</v>
+      </c>
+      <c r="D240" t="n">
+        <v>45</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>4.329999923706055</v>
+      </c>
+      <c r="D241" t="n">
+        <v>61</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>5.920000076293945</v>
+      </c>
+      <c r="D242" t="n">
+        <v>10</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>5.320000171661377</v>
+      </c>
+      <c r="D243" t="n">
+        <v>22</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>19.34000015258789</v>
+      </c>
+      <c r="D244" t="n">
+        <v>49</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>26.20999908447266</v>
+      </c>
+      <c r="D245" t="n">
+        <v>20</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>11.89999961853027</v>
+      </c>
+      <c r="D246" t="n">
+        <v>9</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>4.630000114440918</v>
+      </c>
+      <c r="D247" t="n">
+        <v>26</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>21.70000076293945</v>
+      </c>
+      <c r="D248" t="n">
+        <v>27</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>10.89999961853027</v>
+      </c>
+      <c r="D249" t="n">
+        <v>22</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>4.809999942779541</v>
+      </c>
+      <c r="D250" t="n">
+        <v>20</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>7.300000190734863</v>
+      </c>
+      <c r="D251" t="n">
+        <v>25</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>5.510000228881836</v>
+      </c>
+      <c r="D252" t="n">
+        <v>30</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>45.02000045776367</v>
+      </c>
+      <c r="D253" t="n">
+        <v>23</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>4.400000095367432</v>
+      </c>
+      <c r="D254" t="n">
+        <v>20</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>62.68000030517578</v>
+      </c>
+      <c r="D255" t="n">
+        <v>8</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>49.08000183105469</v>
+      </c>
+      <c r="D256" t="n">
+        <v>16</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>19.60000038146973</v>
+      </c>
+      <c r="D257" t="n">
+        <v>63</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>35.18000030517578</v>
+      </c>
+      <c r="D258" t="n">
+        <v>35</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>106.129997253418</v>
+      </c>
+      <c r="D259" t="n">
+        <v>31</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>45.29999923706055</v>
+      </c>
+      <c r="D260" t="n">
+        <v>11</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>7.46999979019165</v>
+      </c>
+      <c r="D261" t="n">
+        <v>11</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>34.41999816894531</v>
+      </c>
+      <c r="D262" t="n">
+        <v>48</v>
+      </c>
+      <c r="E262" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-02
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E291"/>
+  <dimension ref="A1:E320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5874,7 +5874,7 @@
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="2" t="n">
+      <c r="A263" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B263" t="inlineStr">
@@ -5895,7 +5895,7 @@
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="n">
+      <c r="A264" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B264" t="inlineStr">
@@ -5916,7 +5916,7 @@
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="n">
+      <c r="A265" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B265" t="inlineStr">
@@ -5937,7 +5937,7 @@
       </c>
     </row>
     <row r="266">
-      <c r="A266" s="2" t="n">
+      <c r="A266" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B266" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
     </row>
     <row r="267">
-      <c r="A267" s="2" t="n">
+      <c r="A267" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B267" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="n">
+      <c r="A268" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B268" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="n">
+      <c r="A269" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B269" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="2" t="n">
+      <c r="A270" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B270" t="inlineStr">
@@ -6042,7 +6042,7 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="n">
+      <c r="A271" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B271" t="inlineStr">
@@ -6063,7 +6063,7 @@
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="n">
+      <c r="A272" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B272" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
     </row>
     <row r="273">
-      <c r="A273" s="2" t="n">
+      <c r="A273" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B273" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
     </row>
     <row r="274">
-      <c r="A274" s="2" t="n">
+      <c r="A274" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B274" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="2" t="n">
+      <c r="A275" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B275" t="inlineStr">
@@ -6147,7 +6147,7 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" s="2" t="n">
+      <c r="A276" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B276" t="inlineStr">
@@ -6168,7 +6168,7 @@
       </c>
     </row>
     <row r="277">
-      <c r="A277" s="2" t="n">
+      <c r="A277" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B277" t="inlineStr">
@@ -6189,7 +6189,7 @@
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="2" t="n">
+      <c r="A278" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B278" t="inlineStr">
@@ -6210,7 +6210,7 @@
       </c>
     </row>
     <row r="279">
-      <c r="A279" s="2" t="n">
+      <c r="A279" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B279" t="inlineStr">
@@ -6231,7 +6231,7 @@
       </c>
     </row>
     <row r="280">
-      <c r="A280" s="2" t="n">
+      <c r="A280" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B280" t="inlineStr">
@@ -6252,7 +6252,7 @@
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="n">
+      <c r="A281" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B281" t="inlineStr">
@@ -6273,7 +6273,7 @@
       </c>
     </row>
     <row r="282">
-      <c r="A282" s="2" t="n">
+      <c r="A282" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B282" t="inlineStr">
@@ -6294,7 +6294,7 @@
       </c>
     </row>
     <row r="283">
-      <c r="A283" s="2" t="n">
+      <c r="A283" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B283" t="inlineStr">
@@ -6315,7 +6315,7 @@
       </c>
     </row>
     <row r="284">
-      <c r="A284" s="2" t="n">
+      <c r="A284" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B284" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="2" t="n">
+      <c r="A285" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B285" t="inlineStr">
@@ -6357,7 +6357,7 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" s="2" t="n">
+      <c r="A286" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B286" t="inlineStr">
@@ -6378,7 +6378,7 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="2" t="n">
+      <c r="A287" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B287" t="inlineStr">
@@ -6399,7 +6399,7 @@
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="2" t="n">
+      <c r="A288" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B288" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="2" t="n">
+      <c r="A289" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B289" t="inlineStr">
@@ -6441,7 +6441,7 @@
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="2" t="n">
+      <c r="A290" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B290" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="2" t="n">
+      <c r="A291" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B291" t="inlineStr">
@@ -6477,6 +6477,615 @@
         <v>48</v>
       </c>
       <c r="E291" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>28.6299991607666</v>
+      </c>
+      <c r="D292" t="n">
+        <v>28</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>14.14000034332275</v>
+      </c>
+      <c r="D293" t="n">
+        <v>31</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>22.34000015258789</v>
+      </c>
+      <c r="D294" t="n">
+        <v>30</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>3.849999904632568</v>
+      </c>
+      <c r="D295" t="n">
+        <v>16</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>0.7099999785423279</v>
+      </c>
+      <c r="D296" t="n">
+        <v>12</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>182.5099945068359</v>
+      </c>
+      <c r="D297" t="n">
+        <v>26</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>57.70000076293945</v>
+      </c>
+      <c r="D298" t="n">
+        <v>45</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>4.949999809265137</v>
+      </c>
+      <c r="D299" t="n">
+        <v>61</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>6.369999885559082</v>
+      </c>
+      <c r="D300" t="n">
+        <v>10</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>5.949999809265137</v>
+      </c>
+      <c r="D301" t="n">
+        <v>22</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>19.76000022888184</v>
+      </c>
+      <c r="D302" t="n">
+        <v>49</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>27.39999961853027</v>
+      </c>
+      <c r="D303" t="n">
+        <v>20</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>13.19999980926514</v>
+      </c>
+      <c r="D304" t="n">
+        <v>9</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>4.849999904632568</v>
+      </c>
+      <c r="D305" t="n">
+        <v>26</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>22.39999961853027</v>
+      </c>
+      <c r="D306" t="n">
+        <v>27</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>11.64000034332275</v>
+      </c>
+      <c r="D307" t="n">
+        <v>22</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>5.400000095367432</v>
+      </c>
+      <c r="D308" t="n">
+        <v>20</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>7.849999904632568</v>
+      </c>
+      <c r="D309" t="n">
+        <v>25</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>5.710000038146973</v>
+      </c>
+      <c r="D310" t="n">
+        <v>30</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>48</v>
+      </c>
+      <c r="D311" t="n">
+        <v>23</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>4.619999885559082</v>
+      </c>
+      <c r="D312" t="n">
+        <v>20</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>64.25</v>
+      </c>
+      <c r="D313" t="n">
+        <v>8</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>50.84000015258789</v>
+      </c>
+      <c r="D314" t="n">
+        <v>16</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>20.23999977111816</v>
+      </c>
+      <c r="D315" t="n">
+        <v>63</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>36.97000122070312</v>
+      </c>
+      <c r="D316" t="n">
+        <v>35</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>111.0800018310547</v>
+      </c>
+      <c r="D317" t="n">
+        <v>31</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>46.52000045776367</v>
+      </c>
+      <c r="D318" t="n">
+        <v>11</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>7.840000152587891</v>
+      </c>
+      <c r="D319" t="n">
+        <v>11</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>36.45999908447266</v>
+      </c>
+      <c r="D320" t="n">
+        <v>48</v>
+      </c>
+      <c r="E320" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-03
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E320"/>
+  <dimension ref="A1:E349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6483,7 +6483,7 @@
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="2" t="n">
+      <c r="A292" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B292" t="inlineStr">
@@ -6504,7 +6504,7 @@
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="2" t="n">
+      <c r="A293" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B293" t="inlineStr">
@@ -6525,7 +6525,7 @@
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="2" t="n">
+      <c r="A294" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B294" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="n">
+      <c r="A295" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B295" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="n">
+      <c r="A296" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B296" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="n">
+      <c r="A297" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B297" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
     </row>
     <row r="298">
-      <c r="A298" s="2" t="n">
+      <c r="A298" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B298" t="inlineStr">
@@ -6630,7 +6630,7 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="2" t="n">
+      <c r="A299" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B299" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="2" t="n">
+      <c r="A300" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B300" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="2" t="n">
+      <c r="A301" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B301" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="2" t="n">
+      <c r="A302" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B302" t="inlineStr">
@@ -6714,7 +6714,7 @@
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="2" t="n">
+      <c r="A303" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B303" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="2" t="n">
+      <c r="A304" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B304" t="inlineStr">
@@ -6756,7 +6756,7 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="2" t="n">
+      <c r="A305" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B305" t="inlineStr">
@@ -6777,7 +6777,7 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="2" t="n">
+      <c r="A306" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B306" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="2" t="n">
+      <c r="A307" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B307" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="2" t="n">
+      <c r="A308" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B308" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="2" t="n">
+      <c r="A309" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B309" t="inlineStr">
@@ -6861,7 +6861,7 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="2" t="n">
+      <c r="A310" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B310" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="2" t="n">
+      <c r="A311" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B311" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="2" t="n">
+      <c r="A312" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B312" t="inlineStr">
@@ -6924,7 +6924,7 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="2" t="n">
+      <c r="A313" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B313" t="inlineStr">
@@ -6945,7 +6945,7 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="2" t="n">
+      <c r="A314" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B314" t="inlineStr">
@@ -6966,7 +6966,7 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="2" t="n">
+      <c r="A315" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B315" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="2" t="n">
+      <c r="A316" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B316" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="2" t="n">
+      <c r="A317" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B317" t="inlineStr">
@@ -7029,7 +7029,7 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="2" t="n">
+      <c r="A318" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B318" t="inlineStr">
@@ -7050,7 +7050,7 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="n">
+      <c r="A319" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B319" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="2" t="n">
+      <c r="A320" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="B320" t="inlineStr">
@@ -7086,6 +7086,615 @@
         <v>48</v>
       </c>
       <c r="E320" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>28.98999977111816</v>
+      </c>
+      <c r="D321" t="n">
+        <v>28</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>13.68000030517578</v>
+      </c>
+      <c r="D322" t="n">
+        <v>31</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>22.42000007629395</v>
+      </c>
+      <c r="D323" t="n">
+        <v>30</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>3.799999952316284</v>
+      </c>
+      <c r="D324" t="n">
+        <v>16</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>0.699999988079071</v>
+      </c>
+      <c r="D325" t="n">
+        <v>12</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>182.3000030517578</v>
+      </c>
+      <c r="D326" t="n">
+        <v>26</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>58.4900016784668</v>
+      </c>
+      <c r="D327" t="n">
+        <v>45</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>4.889999866485596</v>
+      </c>
+      <c r="D328" t="n">
+        <v>61</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="D329" t="n">
+        <v>10</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>6.420000076293945</v>
+      </c>
+      <c r="D330" t="n">
+        <v>22</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
+        <v>19.86000061035156</v>
+      </c>
+      <c r="D331" t="n">
+        <v>49</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>27.60000038146973</v>
+      </c>
+      <c r="D332" t="n">
+        <v>20</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>13.22999954223633</v>
+      </c>
+      <c r="D333" t="n">
+        <v>9</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>4.809999942779541</v>
+      </c>
+      <c r="D334" t="n">
+        <v>26</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>22.6299991607666</v>
+      </c>
+      <c r="D335" t="n">
+        <v>27</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>11.78999996185303</v>
+      </c>
+      <c r="D336" t="n">
+        <v>22</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>5.539999961853027</v>
+      </c>
+      <c r="D337" t="n">
+        <v>20</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>7.800000190734863</v>
+      </c>
+      <c r="D338" t="n">
+        <v>25</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
+        <v>5.610000133514404</v>
+      </c>
+      <c r="D339" t="n">
+        <v>30</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>47.56000137329102</v>
+      </c>
+      <c r="D340" t="n">
+        <v>23</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>4.590000152587891</v>
+      </c>
+      <c r="D341" t="n">
+        <v>20</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C342" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="D342" t="n">
+        <v>8</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C343" t="n">
+        <v>51.4900016784668</v>
+      </c>
+      <c r="D343" t="n">
+        <v>16</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C344" t="n">
+        <v>20.19000053405762</v>
+      </c>
+      <c r="D344" t="n">
+        <v>63</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C345" t="n">
+        <v>37.45000076293945</v>
+      </c>
+      <c r="D345" t="n">
+        <v>35</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C346" t="n">
+        <v>111.2699966430664</v>
+      </c>
+      <c r="D346" t="n">
+        <v>31</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C347" t="n">
+        <v>46.65000152587891</v>
+      </c>
+      <c r="D347" t="n">
+        <v>11</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C348" t="n">
+        <v>7.840000152587891</v>
+      </c>
+      <c r="D348" t="n">
+        <v>11</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C349" t="n">
+        <v>36.72999954223633</v>
+      </c>
+      <c r="D349" t="n">
+        <v>48</v>
+      </c>
+      <c r="E349" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-04
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7092,7 +7092,7 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="2" t="n">
+      <c r="A321" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B321" t="inlineStr">
@@ -7113,7 +7113,7 @@
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="2" t="n">
+      <c r="A322" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B322" t="inlineStr">
@@ -7134,7 +7134,7 @@
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="2" t="n">
+      <c r="A323" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B323" t="inlineStr">
@@ -7155,7 +7155,7 @@
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="2" t="n">
+      <c r="A324" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B324" t="inlineStr">
@@ -7176,7 +7176,7 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="2" t="n">
+      <c r="A325" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B325" t="inlineStr">
@@ -7197,7 +7197,7 @@
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="2" t="n">
+      <c r="A326" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B326" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="2" t="n">
+      <c r="A327" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B327" t="inlineStr">
@@ -7239,7 +7239,7 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="2" t="n">
+      <c r="A328" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B328" t="inlineStr">
@@ -7260,7 +7260,7 @@
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="2" t="n">
+      <c r="A329" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B329" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="2" t="n">
+      <c r="A330" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B330" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="n">
+      <c r="A331" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B331" t="inlineStr">
@@ -7323,7 +7323,7 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="n">
+      <c r="A332" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B332" t="inlineStr">
@@ -7344,7 +7344,7 @@
       </c>
     </row>
     <row r="333">
-      <c r="A333" s="2" t="n">
+      <c r="A333" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B333" t="inlineStr">
@@ -7365,7 +7365,7 @@
       </c>
     </row>
     <row r="334">
-      <c r="A334" s="2" t="n">
+      <c r="A334" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B334" t="inlineStr">
@@ -7386,7 +7386,7 @@
       </c>
     </row>
     <row r="335">
-      <c r="A335" s="2" t="n">
+      <c r="A335" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B335" t="inlineStr">
@@ -7407,7 +7407,7 @@
       </c>
     </row>
     <row r="336">
-      <c r="A336" s="2" t="n">
+      <c r="A336" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B336" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" s="2" t="n">
+      <c r="A337" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B337" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
     </row>
     <row r="338">
-      <c r="A338" s="2" t="n">
+      <c r="A338" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B338" t="inlineStr">
@@ -7470,7 +7470,7 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="2" t="n">
+      <c r="A339" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B339" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
     </row>
     <row r="340">
-      <c r="A340" s="2" t="n">
+      <c r="A340" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B340" t="inlineStr">
@@ -7512,7 +7512,7 @@
       </c>
     </row>
     <row r="341">
-      <c r="A341" s="2" t="n">
+      <c r="A341" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B341" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
     </row>
     <row r="342">
-      <c r="A342" s="2" t="n">
+      <c r="A342" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B342" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
     </row>
     <row r="343">
-      <c r="A343" s="2" t="n">
+      <c r="A343" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B343" t="inlineStr">
@@ -7575,7 +7575,7 @@
       </c>
     </row>
     <row r="344">
-      <c r="A344" s="2" t="n">
+      <c r="A344" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B344" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
     </row>
     <row r="345">
-      <c r="A345" s="2" t="n">
+      <c r="A345" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B345" t="inlineStr">
@@ -7617,7 +7617,7 @@
       </c>
     </row>
     <row r="346">
-      <c r="A346" s="2" t="n">
+      <c r="A346" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B346" t="inlineStr">
@@ -7638,7 +7638,7 @@
       </c>
     </row>
     <row r="347">
-      <c r="A347" s="2" t="n">
+      <c r="A347" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B347" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
     </row>
     <row r="348">
-      <c r="A348" s="2" t="n">
+      <c r="A348" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B348" t="inlineStr">
@@ -7680,7 +7680,7 @@
       </c>
     </row>
     <row r="349">
-      <c r="A349" s="2" t="n">
+      <c r="A349" s="1" t="n">
         <v>46268</v>
       </c>
       <c r="B349" t="inlineStr">
@@ -7695,6 +7695,615 @@
         <v>48</v>
       </c>
       <c r="E349" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C350" t="n">
+        <v>28.81999969482422</v>
+      </c>
+      <c r="D350" t="n">
+        <v>28</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C351" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D351" t="n">
+        <v>31</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C352" t="n">
+        <v>22.45000076293945</v>
+      </c>
+      <c r="D352" t="n">
+        <v>30</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C353" t="n">
+        <v>3.970000028610229</v>
+      </c>
+      <c r="D353" t="n">
+        <v>16</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C354" t="n">
+        <v>0.6899999976158142</v>
+      </c>
+      <c r="D354" t="n">
+        <v>12</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>182.0200042724609</v>
+      </c>
+      <c r="D355" t="n">
+        <v>26</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C356" t="n">
+        <v>58.88000106811523</v>
+      </c>
+      <c r="D356" t="n">
+        <v>45</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>4.800000190734863</v>
+      </c>
+      <c r="D357" t="n">
+        <v>61</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>6.650000095367432</v>
+      </c>
+      <c r="D358" t="n">
+        <v>10</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>6.320000171661377</v>
+      </c>
+      <c r="D359" t="n">
+        <v>22</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>19.86000061035156</v>
+      </c>
+      <c r="D360" t="n">
+        <v>49</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>27.57999992370605</v>
+      </c>
+      <c r="D361" t="n">
+        <v>20</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>12.94999980926514</v>
+      </c>
+      <c r="D362" t="n">
+        <v>9</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>4.889999866485596</v>
+      </c>
+      <c r="D363" t="n">
+        <v>26</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>23.11000061035156</v>
+      </c>
+      <c r="D364" t="n">
+        <v>27</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>11.46000003814697</v>
+      </c>
+      <c r="D365" t="n">
+        <v>22</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>5.739999771118164</v>
+      </c>
+      <c r="D366" t="n">
+        <v>20</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>8.039999961853027</v>
+      </c>
+      <c r="D367" t="n">
+        <v>25</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>5.570000171661377</v>
+      </c>
+      <c r="D368" t="n">
+        <v>30</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>46.91999816894531</v>
+      </c>
+      <c r="D369" t="n">
+        <v>23</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>4.550000190734863</v>
+      </c>
+      <c r="D370" t="n">
+        <v>20</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>60.22999954223633</v>
+      </c>
+      <c r="D371" t="n">
+        <v>8</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>51.56000137329102</v>
+      </c>
+      <c r="D372" t="n">
+        <v>16</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>20.04999923706055</v>
+      </c>
+      <c r="D373" t="n">
+        <v>63</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>37.13000106811523</v>
+      </c>
+      <c r="D374" t="n">
+        <v>35</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>111.1699981689453</v>
+      </c>
+      <c r="D375" t="n">
+        <v>31</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>46.7599983215332</v>
+      </c>
+      <c r="D376" t="n">
+        <v>11</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>7.670000076293945</v>
+      </c>
+      <c r="D377" t="n">
+        <v>11</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>36.7599983215332</v>
+      </c>
+      <c r="D378" t="n">
+        <v>48</v>
+      </c>
+      <c r="E378" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-07
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E378"/>
+  <dimension ref="A1:E407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7701,7 +7701,7 @@
       </c>
     </row>
     <row r="350">
-      <c r="A350" s="2" t="n">
+      <c r="A350" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B350" t="inlineStr">
@@ -7722,7 +7722,7 @@
       </c>
     </row>
     <row r="351">
-      <c r="A351" s="2" t="n">
+      <c r="A351" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B351" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
     </row>
     <row r="352">
-      <c r="A352" s="2" t="n">
+      <c r="A352" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B352" t="inlineStr">
@@ -7764,7 +7764,7 @@
       </c>
     </row>
     <row r="353">
-      <c r="A353" s="2" t="n">
+      <c r="A353" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B353" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
     </row>
     <row r="354">
-      <c r="A354" s="2" t="n">
+      <c r="A354" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B354" t="inlineStr">
@@ -7806,7 +7806,7 @@
       </c>
     </row>
     <row r="355">
-      <c r="A355" s="2" t="n">
+      <c r="A355" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B355" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
     </row>
     <row r="356">
-      <c r="A356" s="2" t="n">
+      <c r="A356" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B356" t="inlineStr">
@@ -7848,7 +7848,7 @@
       </c>
     </row>
     <row r="357">
-      <c r="A357" s="2" t="n">
+      <c r="A357" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B357" t="inlineStr">
@@ -7869,7 +7869,7 @@
       </c>
     </row>
     <row r="358">
-      <c r="A358" s="2" t="n">
+      <c r="A358" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B358" t="inlineStr">
@@ -7890,7 +7890,7 @@
       </c>
     </row>
     <row r="359">
-      <c r="A359" s="2" t="n">
+      <c r="A359" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B359" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
     </row>
     <row r="360">
-      <c r="A360" s="2" t="n">
+      <c r="A360" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B360" t="inlineStr">
@@ -7932,7 +7932,7 @@
       </c>
     </row>
     <row r="361">
-      <c r="A361" s="2" t="n">
+      <c r="A361" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B361" t="inlineStr">
@@ -7953,7 +7953,7 @@
       </c>
     </row>
     <row r="362">
-      <c r="A362" s="2" t="n">
+      <c r="A362" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B362" t="inlineStr">
@@ -7974,7 +7974,7 @@
       </c>
     </row>
     <row r="363">
-      <c r="A363" s="2" t="n">
+      <c r="A363" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B363" t="inlineStr">
@@ -7995,7 +7995,7 @@
       </c>
     </row>
     <row r="364">
-      <c r="A364" s="2" t="n">
+      <c r="A364" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B364" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
     </row>
     <row r="365">
-      <c r="A365" s="2" t="n">
+      <c r="A365" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B365" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
     </row>
     <row r="366">
-      <c r="A366" s="2" t="n">
+      <c r="A366" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B366" t="inlineStr">
@@ -8058,7 +8058,7 @@
       </c>
     </row>
     <row r="367">
-      <c r="A367" s="2" t="n">
+      <c r="A367" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B367" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
     </row>
     <row r="368">
-      <c r="A368" s="2" t="n">
+      <c r="A368" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B368" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
     </row>
     <row r="369">
-      <c r="A369" s="2" t="n">
+      <c r="A369" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B369" t="inlineStr">
@@ -8121,7 +8121,7 @@
       </c>
     </row>
     <row r="370">
-      <c r="A370" s="2" t="n">
+      <c r="A370" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B370" t="inlineStr">
@@ -8142,7 +8142,7 @@
       </c>
     </row>
     <row r="371">
-      <c r="A371" s="2" t="n">
+      <c r="A371" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B371" t="inlineStr">
@@ -8163,7 +8163,7 @@
       </c>
     </row>
     <row r="372">
-      <c r="A372" s="2" t="n">
+      <c r="A372" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B372" t="inlineStr">
@@ -8184,7 +8184,7 @@
       </c>
     </row>
     <row r="373">
-      <c r="A373" s="2" t="n">
+      <c r="A373" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B373" t="inlineStr">
@@ -8205,7 +8205,7 @@
       </c>
     </row>
     <row r="374">
-      <c r="A374" s="2" t="n">
+      <c r="A374" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B374" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
     </row>
     <row r="375">
-      <c r="A375" s="2" t="n">
+      <c r="A375" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B375" t="inlineStr">
@@ -8247,7 +8247,7 @@
       </c>
     </row>
     <row r="376">
-      <c r="A376" s="2" t="n">
+      <c r="A376" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B376" t="inlineStr">
@@ -8268,7 +8268,7 @@
       </c>
     </row>
     <row r="377">
-      <c r="A377" s="2" t="n">
+      <c r="A377" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B377" t="inlineStr">
@@ -8289,7 +8289,7 @@
       </c>
     </row>
     <row r="378">
-      <c r="A378" s="2" t="n">
+      <c r="A378" s="1" t="n">
         <v>46269</v>
       </c>
       <c r="B378" t="inlineStr">
@@ -8304,6 +8304,615 @@
         <v>48</v>
       </c>
       <c r="E378" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>28.80999946594238</v>
+      </c>
+      <c r="D379" t="n">
+        <v>28</v>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>13.56999969482422</v>
+      </c>
+      <c r="D380" t="n">
+        <v>31</v>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>22.52000045776367</v>
+      </c>
+      <c r="D381" t="n">
+        <v>30</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>3.950000047683716</v>
+      </c>
+      <c r="D382" t="n">
+        <v>16</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>0.6899999976158142</v>
+      </c>
+      <c r="D383" t="n">
+        <v>12</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>181.9400024414062</v>
+      </c>
+      <c r="D384" t="n">
+        <v>26</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>59.2400016784668</v>
+      </c>
+      <c r="D385" t="n">
+        <v>45</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>4.800000190734863</v>
+      </c>
+      <c r="D386" t="n">
+        <v>61</v>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>6.590000152587891</v>
+      </c>
+      <c r="D387" t="n">
+        <v>10</v>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C388" t="n">
+        <v>6.360000133514404</v>
+      </c>
+      <c r="D388" t="n">
+        <v>22</v>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C389" t="n">
+        <v>19.97999954223633</v>
+      </c>
+      <c r="D389" t="n">
+        <v>49</v>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C390" t="n">
+        <v>27.59000015258789</v>
+      </c>
+      <c r="D390" t="n">
+        <v>20</v>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C391" t="n">
+        <v>13</v>
+      </c>
+      <c r="D391" t="n">
+        <v>9</v>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C392" t="n">
+        <v>4.869999885559082</v>
+      </c>
+      <c r="D392" t="n">
+        <v>26</v>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C393" t="n">
+        <v>23.15999984741211</v>
+      </c>
+      <c r="D393" t="n">
+        <v>27</v>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C394" t="n">
+        <v>11.44999980926514</v>
+      </c>
+      <c r="D394" t="n">
+        <v>22</v>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>5.789999961853027</v>
+      </c>
+      <c r="D395" t="n">
+        <v>20</v>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>8.109999656677246</v>
+      </c>
+      <c r="D396" t="n">
+        <v>25</v>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>5.550000190734863</v>
+      </c>
+      <c r="D397" t="n">
+        <v>30</v>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>47.11000061035156</v>
+      </c>
+      <c r="D398" t="n">
+        <v>23</v>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C399" t="n">
+        <v>4.579999923706055</v>
+      </c>
+      <c r="D399" t="n">
+        <v>20</v>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>60.18999862670898</v>
+      </c>
+      <c r="D400" t="n">
+        <v>8</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>51.65999984741211</v>
+      </c>
+      <c r="D401" t="n">
+        <v>16</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>19.98999977111816</v>
+      </c>
+      <c r="D402" t="n">
+        <v>63</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C403" t="n">
+        <v>37.13000106811523</v>
+      </c>
+      <c r="D403" t="n">
+        <v>35</v>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C404" t="n">
+        <v>110.9899978637695</v>
+      </c>
+      <c r="D404" t="n">
+        <v>31</v>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>46.88999938964844</v>
+      </c>
+      <c r="D405" t="n">
+        <v>11</v>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>7.630000114440918</v>
+      </c>
+      <c r="D406" t="n">
+        <v>11</v>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>36.9900016784668</v>
+      </c>
+      <c r="D407" t="n">
+        <v>48</v>
+      </c>
+      <c r="E407" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-08
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E407"/>
+  <dimension ref="A1:E436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8310,7 +8310,7 @@
       </c>
     </row>
     <row r="379">
-      <c r="A379" s="2" t="n">
+      <c r="A379" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B379" t="inlineStr">
@@ -8331,7 +8331,7 @@
       </c>
     </row>
     <row r="380">
-      <c r="A380" s="2" t="n">
+      <c r="A380" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B380" t="inlineStr">
@@ -8352,7 +8352,7 @@
       </c>
     </row>
     <row r="381">
-      <c r="A381" s="2" t="n">
+      <c r="A381" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B381" t="inlineStr">
@@ -8373,7 +8373,7 @@
       </c>
     </row>
     <row r="382">
-      <c r="A382" s="2" t="n">
+      <c r="A382" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B382" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
     </row>
     <row r="383">
-      <c r="A383" s="2" t="n">
+      <c r="A383" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B383" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
     </row>
     <row r="384">
-      <c r="A384" s="2" t="n">
+      <c r="A384" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B384" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
     </row>
     <row r="385">
-      <c r="A385" s="2" t="n">
+      <c r="A385" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B385" t="inlineStr">
@@ -8457,7 +8457,7 @@
       </c>
     </row>
     <row r="386">
-      <c r="A386" s="2" t="n">
+      <c r="A386" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B386" t="inlineStr">
@@ -8478,7 +8478,7 @@
       </c>
     </row>
     <row r="387">
-      <c r="A387" s="2" t="n">
+      <c r="A387" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B387" t="inlineStr">
@@ -8499,7 +8499,7 @@
       </c>
     </row>
     <row r="388">
-      <c r="A388" s="2" t="n">
+      <c r="A388" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B388" t="inlineStr">
@@ -8520,7 +8520,7 @@
       </c>
     </row>
     <row r="389">
-      <c r="A389" s="2" t="n">
+      <c r="A389" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B389" t="inlineStr">
@@ -8541,7 +8541,7 @@
       </c>
     </row>
     <row r="390">
-      <c r="A390" s="2" t="n">
+      <c r="A390" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B390" t="inlineStr">
@@ -8562,7 +8562,7 @@
       </c>
     </row>
     <row r="391">
-      <c r="A391" s="2" t="n">
+      <c r="A391" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B391" t="inlineStr">
@@ -8583,7 +8583,7 @@
       </c>
     </row>
     <row r="392">
-      <c r="A392" s="2" t="n">
+      <c r="A392" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B392" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
     </row>
     <row r="393">
-      <c r="A393" s="2" t="n">
+      <c r="A393" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B393" t="inlineStr">
@@ -8625,7 +8625,7 @@
       </c>
     </row>
     <row r="394">
-      <c r="A394" s="2" t="n">
+      <c r="A394" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B394" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
     </row>
     <row r="395">
-      <c r="A395" s="2" t="n">
+      <c r="A395" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B395" t="inlineStr">
@@ -8667,7 +8667,7 @@
       </c>
     </row>
     <row r="396">
-      <c r="A396" s="2" t="n">
+      <c r="A396" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B396" t="inlineStr">
@@ -8688,7 +8688,7 @@
       </c>
     </row>
     <row r="397">
-      <c r="A397" s="2" t="n">
+      <c r="A397" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B397" t="inlineStr">
@@ -8709,7 +8709,7 @@
       </c>
     </row>
     <row r="398">
-      <c r="A398" s="2" t="n">
+      <c r="A398" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B398" t="inlineStr">
@@ -8730,7 +8730,7 @@
       </c>
     </row>
     <row r="399">
-      <c r="A399" s="2" t="n">
+      <c r="A399" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B399" t="inlineStr">
@@ -8751,7 +8751,7 @@
       </c>
     </row>
     <row r="400">
-      <c r="A400" s="2" t="n">
+      <c r="A400" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B400" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
     </row>
     <row r="401">
-      <c r="A401" s="2" t="n">
+      <c r="A401" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B401" t="inlineStr">
@@ -8793,7 +8793,7 @@
       </c>
     </row>
     <row r="402">
-      <c r="A402" s="2" t="n">
+      <c r="A402" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B402" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
     </row>
     <row r="403">
-      <c r="A403" s="2" t="n">
+      <c r="A403" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B403" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
     </row>
     <row r="404">
-      <c r="A404" s="2" t="n">
+      <c r="A404" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B404" t="inlineStr">
@@ -8856,7 +8856,7 @@
       </c>
     </row>
     <row r="405">
-      <c r="A405" s="2" t="n">
+      <c r="A405" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B405" t="inlineStr">
@@ -8877,7 +8877,7 @@
       </c>
     </row>
     <row r="406">
-      <c r="A406" s="2" t="n">
+      <c r="A406" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B406" t="inlineStr">
@@ -8898,7 +8898,7 @@
       </c>
     </row>
     <row r="407">
-      <c r="A407" s="2" t="n">
+      <c r="A407" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="B407" t="inlineStr">
@@ -8913,6 +8913,615 @@
         <v>48</v>
       </c>
       <c r="E407" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>29.1299991607666</v>
+      </c>
+      <c r="D408" t="n">
+        <v>28</v>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>13.02999973297119</v>
+      </c>
+      <c r="D409" t="n">
+        <v>31</v>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>22.64999961853027</v>
+      </c>
+      <c r="D410" t="n">
+        <v>30</v>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C411" t="n">
+        <v>3.940000057220459</v>
+      </c>
+      <c r="D411" t="n">
+        <v>16</v>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>0.6399999856948853</v>
+      </c>
+      <c r="D412" t="n">
+        <v>12</v>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>184.6999969482422</v>
+      </c>
+      <c r="D413" t="n">
+        <v>26</v>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>60.72000122070312</v>
+      </c>
+      <c r="D414" t="n">
+        <v>45</v>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>4.909999847412109</v>
+      </c>
+      <c r="D415" t="n">
+        <v>61</v>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>6.690000057220459</v>
+      </c>
+      <c r="D416" t="n">
+        <v>10</v>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>6.579999923706055</v>
+      </c>
+      <c r="D417" t="n">
+        <v>22</v>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>20.20999908447266</v>
+      </c>
+      <c r="D418" t="n">
+        <v>49</v>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>27.76000022888184</v>
+      </c>
+      <c r="D419" t="n">
+        <v>20</v>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>12.92000007629395</v>
+      </c>
+      <c r="D420" t="n">
+        <v>9</v>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>4.809999942779541</v>
+      </c>
+      <c r="D421" t="n">
+        <v>26</v>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C422" t="n">
+        <v>23.10000038146973</v>
+      </c>
+      <c r="D422" t="n">
+        <v>27</v>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>11.64000034332275</v>
+      </c>
+      <c r="D423" t="n">
+        <v>22</v>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>5.820000171661377</v>
+      </c>
+      <c r="D424" t="n">
+        <v>20</v>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>8.180000305175781</v>
+      </c>
+      <c r="D425" t="n">
+        <v>25</v>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>5.800000190734863</v>
+      </c>
+      <c r="D426" t="n">
+        <v>30</v>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C427" t="n">
+        <v>48.08000183105469</v>
+      </c>
+      <c r="D427" t="n">
+        <v>23</v>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C428" t="n">
+        <v>4.590000152587891</v>
+      </c>
+      <c r="D428" t="n">
+        <v>20</v>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C429" t="n">
+        <v>62.15999984741211</v>
+      </c>
+      <c r="D429" t="n">
+        <v>8</v>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C430" t="n">
+        <v>51.20000076293945</v>
+      </c>
+      <c r="D430" t="n">
+        <v>16</v>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C431" t="n">
+        <v>20.1299991607666</v>
+      </c>
+      <c r="D431" t="n">
+        <v>63</v>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C432" t="n">
+        <v>37.63000106811523</v>
+      </c>
+      <c r="D432" t="n">
+        <v>35</v>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C433" t="n">
+        <v>112.0500030517578</v>
+      </c>
+      <c r="D433" t="n">
+        <v>31</v>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C434" t="n">
+        <v>46.97999954223633</v>
+      </c>
+      <c r="D434" t="n">
+        <v>11</v>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C435" t="n">
+        <v>7.539999961853027</v>
+      </c>
+      <c r="D435" t="n">
+        <v>11</v>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C436" t="n">
+        <v>37.34000015258789</v>
+      </c>
+      <c r="D436" t="n">
+        <v>48</v>
+      </c>
+      <c r="E436" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-09
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E436"/>
+  <dimension ref="A1:E465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8919,7 +8919,7 @@
       </c>
     </row>
     <row r="408">
-      <c r="A408" s="2" t="n">
+      <c r="A408" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B408" t="inlineStr">
@@ -8940,7 +8940,7 @@
       </c>
     </row>
     <row r="409">
-      <c r="A409" s="2" t="n">
+      <c r="A409" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B409" t="inlineStr">
@@ -8961,7 +8961,7 @@
       </c>
     </row>
     <row r="410">
-      <c r="A410" s="2" t="n">
+      <c r="A410" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B410" t="inlineStr">
@@ -8982,7 +8982,7 @@
       </c>
     </row>
     <row r="411">
-      <c r="A411" s="2" t="n">
+      <c r="A411" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B411" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
     </row>
     <row r="412">
-      <c r="A412" s="2" t="n">
+      <c r="A412" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B412" t="inlineStr">
@@ -9024,7 +9024,7 @@
       </c>
     </row>
     <row r="413">
-      <c r="A413" s="2" t="n">
+      <c r="A413" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B413" t="inlineStr">
@@ -9045,7 +9045,7 @@
       </c>
     </row>
     <row r="414">
-      <c r="A414" s="2" t="n">
+      <c r="A414" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B414" t="inlineStr">
@@ -9066,7 +9066,7 @@
       </c>
     </row>
     <row r="415">
-      <c r="A415" s="2" t="n">
+      <c r="A415" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B415" t="inlineStr">
@@ -9087,7 +9087,7 @@
       </c>
     </row>
     <row r="416">
-      <c r="A416" s="2" t="n">
+      <c r="A416" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B416" t="inlineStr">
@@ -9108,7 +9108,7 @@
       </c>
     </row>
     <row r="417">
-      <c r="A417" s="2" t="n">
+      <c r="A417" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B417" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
     </row>
     <row r="418">
-      <c r="A418" s="2" t="n">
+      <c r="A418" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B418" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
     </row>
     <row r="419">
-      <c r="A419" s="2" t="n">
+      <c r="A419" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B419" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
     </row>
     <row r="420">
-      <c r="A420" s="2" t="n">
+      <c r="A420" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B420" t="inlineStr">
@@ -9192,7 +9192,7 @@
       </c>
     </row>
     <row r="421">
-      <c r="A421" s="2" t="n">
+      <c r="A421" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B421" t="inlineStr">
@@ -9213,7 +9213,7 @@
       </c>
     </row>
     <row r="422">
-      <c r="A422" s="2" t="n">
+      <c r="A422" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B422" t="inlineStr">
@@ -9234,7 +9234,7 @@
       </c>
     </row>
     <row r="423">
-      <c r="A423" s="2" t="n">
+      <c r="A423" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B423" t="inlineStr">
@@ -9255,7 +9255,7 @@
       </c>
     </row>
     <row r="424">
-      <c r="A424" s="2" t="n">
+      <c r="A424" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B424" t="inlineStr">
@@ -9276,7 +9276,7 @@
       </c>
     </row>
     <row r="425">
-      <c r="A425" s="2" t="n">
+      <c r="A425" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B425" t="inlineStr">
@@ -9297,7 +9297,7 @@
       </c>
     </row>
     <row r="426">
-      <c r="A426" s="2" t="n">
+      <c r="A426" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B426" t="inlineStr">
@@ -9318,7 +9318,7 @@
       </c>
     </row>
     <row r="427">
-      <c r="A427" s="2" t="n">
+      <c r="A427" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B427" t="inlineStr">
@@ -9339,7 +9339,7 @@
       </c>
     </row>
     <row r="428">
-      <c r="A428" s="2" t="n">
+      <c r="A428" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B428" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
     </row>
     <row r="429">
-      <c r="A429" s="2" t="n">
+      <c r="A429" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B429" t="inlineStr">
@@ -9381,7 +9381,7 @@
       </c>
     </row>
     <row r="430">
-      <c r="A430" s="2" t="n">
+      <c r="A430" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B430" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
     </row>
     <row r="431">
-      <c r="A431" s="2" t="n">
+      <c r="A431" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B431" t="inlineStr">
@@ -9423,7 +9423,7 @@
       </c>
     </row>
     <row r="432">
-      <c r="A432" s="2" t="n">
+      <c r="A432" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B432" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
     </row>
     <row r="433">
-      <c r="A433" s="2" t="n">
+      <c r="A433" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B433" t="inlineStr">
@@ -9465,7 +9465,7 @@
       </c>
     </row>
     <row r="434">
-      <c r="A434" s="2" t="n">
+      <c r="A434" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B434" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
     </row>
     <row r="435">
-      <c r="A435" s="2" t="n">
+      <c r="A435" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B435" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
     </row>
     <row r="436">
-      <c r="A436" s="2" t="n">
+      <c r="A436" s="1" t="n">
         <v>46273</v>
       </c>
       <c r="B436" t="inlineStr">
@@ -9522,6 +9522,615 @@
         <v>48</v>
       </c>
       <c r="E436" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C437" t="n">
+        <v>28.45999908447266</v>
+      </c>
+      <c r="D437" t="n">
+        <v>28</v>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C438" t="n">
+        <v>13.26000022888184</v>
+      </c>
+      <c r="D438" t="n">
+        <v>31</v>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C439" t="n">
+        <v>22.1200008392334</v>
+      </c>
+      <c r="D439" t="n">
+        <v>30</v>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C440" t="n">
+        <v>3.950000047683716</v>
+      </c>
+      <c r="D440" t="n">
+        <v>16</v>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C441" t="n">
+        <v>0.6399999856948853</v>
+      </c>
+      <c r="D441" t="n">
+        <v>12</v>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C442" t="n">
+        <v>182.8500061035156</v>
+      </c>
+      <c r="D442" t="n">
+        <v>26</v>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C443" t="n">
+        <v>58.79999923706055</v>
+      </c>
+      <c r="D443" t="n">
+        <v>45</v>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C444" t="n">
+        <v>4.989999771118164</v>
+      </c>
+      <c r="D444" t="n">
+        <v>61</v>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C445" t="n">
+        <v>6.929999828338623</v>
+      </c>
+      <c r="D445" t="n">
+        <v>10</v>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C446" t="n">
+        <v>7.03000020980835</v>
+      </c>
+      <c r="D446" t="n">
+        <v>22</v>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C447" t="n">
+        <v>19.84000015258789</v>
+      </c>
+      <c r="D447" t="n">
+        <v>49</v>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C448" t="n">
+        <v>27.26000022888184</v>
+      </c>
+      <c r="D448" t="n">
+        <v>20</v>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C449" t="n">
+        <v>12.8100004196167</v>
+      </c>
+      <c r="D449" t="n">
+        <v>9</v>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C450" t="n">
+        <v>4.699999809265137</v>
+      </c>
+      <c r="D450" t="n">
+        <v>26</v>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C451" t="n">
+        <v>22.54999923706055</v>
+      </c>
+      <c r="D451" t="n">
+        <v>27</v>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C452" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D452" t="n">
+        <v>22</v>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C453" t="n">
+        <v>5.579999923706055</v>
+      </c>
+      <c r="D453" t="n">
+        <v>20</v>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C454" t="n">
+        <v>7.710000038146973</v>
+      </c>
+      <c r="D454" t="n">
+        <v>25</v>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C455" t="n">
+        <v>5.619999885559082</v>
+      </c>
+      <c r="D455" t="n">
+        <v>30</v>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C456" t="n">
+        <v>48.52999877929688</v>
+      </c>
+      <c r="D456" t="n">
+        <v>23</v>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C457" t="n">
+        <v>4.460000038146973</v>
+      </c>
+      <c r="D457" t="n">
+        <v>20</v>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C458" t="n">
+        <v>62.59999847412109</v>
+      </c>
+      <c r="D458" t="n">
+        <v>8</v>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C459" t="n">
+        <v>50.61999893188477</v>
+      </c>
+      <c r="D459" t="n">
+        <v>16</v>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C460" t="n">
+        <v>19.61000061035156</v>
+      </c>
+      <c r="D460" t="n">
+        <v>63</v>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>36.86999893188477</v>
+      </c>
+      <c r="D461" t="n">
+        <v>35</v>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C462" t="n">
+        <v>110.2399978637695</v>
+      </c>
+      <c r="D462" t="n">
+        <v>31</v>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C463" t="n">
+        <v>47.38000106811523</v>
+      </c>
+      <c r="D463" t="n">
+        <v>11</v>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C464" t="n">
+        <v>7.619999885559082</v>
+      </c>
+      <c r="D464" t="n">
+        <v>11</v>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C465" t="n">
+        <v>37.81999969482422</v>
+      </c>
+      <c r="D465" t="n">
+        <v>48</v>
+      </c>
+      <c r="E465" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-10
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E465"/>
+  <dimension ref="A1:E494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9528,7 +9528,7 @@
       </c>
     </row>
     <row r="437">
-      <c r="A437" s="2" t="n">
+      <c r="A437" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B437" t="inlineStr">
@@ -9549,7 +9549,7 @@
       </c>
     </row>
     <row r="438">
-      <c r="A438" s="2" t="n">
+      <c r="A438" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B438" t="inlineStr">
@@ -9570,7 +9570,7 @@
       </c>
     </row>
     <row r="439">
-      <c r="A439" s="2" t="n">
+      <c r="A439" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B439" t="inlineStr">
@@ -9591,7 +9591,7 @@
       </c>
     </row>
     <row r="440">
-      <c r="A440" s="2" t="n">
+      <c r="A440" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B440" t="inlineStr">
@@ -9612,7 +9612,7 @@
       </c>
     </row>
     <row r="441">
-      <c r="A441" s="2" t="n">
+      <c r="A441" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B441" t="inlineStr">
@@ -9633,7 +9633,7 @@
       </c>
     </row>
     <row r="442">
-      <c r="A442" s="2" t="n">
+      <c r="A442" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B442" t="inlineStr">
@@ -9654,7 +9654,7 @@
       </c>
     </row>
     <row r="443">
-      <c r="A443" s="2" t="n">
+      <c r="A443" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B443" t="inlineStr">
@@ -9675,7 +9675,7 @@
       </c>
     </row>
     <row r="444">
-      <c r="A444" s="2" t="n">
+      <c r="A444" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B444" t="inlineStr">
@@ -9696,7 +9696,7 @@
       </c>
     </row>
     <row r="445">
-      <c r="A445" s="2" t="n">
+      <c r="A445" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B445" t="inlineStr">
@@ -9717,7 +9717,7 @@
       </c>
     </row>
     <row r="446">
-      <c r="A446" s="2" t="n">
+      <c r="A446" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B446" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
     </row>
     <row r="447">
-      <c r="A447" s="2" t="n">
+      <c r="A447" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B447" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
     </row>
     <row r="448">
-      <c r="A448" s="2" t="n">
+      <c r="A448" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B448" t="inlineStr">
@@ -9780,7 +9780,7 @@
       </c>
     </row>
     <row r="449">
-      <c r="A449" s="2" t="n">
+      <c r="A449" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B449" t="inlineStr">
@@ -9801,7 +9801,7 @@
       </c>
     </row>
     <row r="450">
-      <c r="A450" s="2" t="n">
+      <c r="A450" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B450" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
     </row>
     <row r="451">
-      <c r="A451" s="2" t="n">
+      <c r="A451" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B451" t="inlineStr">
@@ -9843,7 +9843,7 @@
       </c>
     </row>
     <row r="452">
-      <c r="A452" s="2" t="n">
+      <c r="A452" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B452" t="inlineStr">
@@ -9864,7 +9864,7 @@
       </c>
     </row>
     <row r="453">
-      <c r="A453" s="2" t="n">
+      <c r="A453" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B453" t="inlineStr">
@@ -9885,7 +9885,7 @@
       </c>
     </row>
     <row r="454">
-      <c r="A454" s="2" t="n">
+      <c r="A454" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B454" t="inlineStr">
@@ -9906,7 +9906,7 @@
       </c>
     </row>
     <row r="455">
-      <c r="A455" s="2" t="n">
+      <c r="A455" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B455" t="inlineStr">
@@ -9927,7 +9927,7 @@
       </c>
     </row>
     <row r="456">
-      <c r="A456" s="2" t="n">
+      <c r="A456" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B456" t="inlineStr">
@@ -9948,7 +9948,7 @@
       </c>
     </row>
     <row r="457">
-      <c r="A457" s="2" t="n">
+      <c r="A457" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B457" t="inlineStr">
@@ -9969,7 +9969,7 @@
       </c>
     </row>
     <row r="458">
-      <c r="A458" s="2" t="n">
+      <c r="A458" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B458" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
     </row>
     <row r="459">
-      <c r="A459" s="2" t="n">
+      <c r="A459" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B459" t="inlineStr">
@@ -10011,7 +10011,7 @@
       </c>
     </row>
     <row r="460">
-      <c r="A460" s="2" t="n">
+      <c r="A460" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B460" t="inlineStr">
@@ -10032,7 +10032,7 @@
       </c>
     </row>
     <row r="461">
-      <c r="A461" s="2" t="n">
+      <c r="A461" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B461" t="inlineStr">
@@ -10053,7 +10053,7 @@
       </c>
     </row>
     <row r="462">
-      <c r="A462" s="2" t="n">
+      <c r="A462" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B462" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
     </row>
     <row r="463">
-      <c r="A463" s="2" t="n">
+      <c r="A463" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B463" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
     </row>
     <row r="464">
-      <c r="A464" s="2" t="n">
+      <c r="A464" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B464" t="inlineStr">
@@ -10116,7 +10116,7 @@
       </c>
     </row>
     <row r="465">
-      <c r="A465" s="2" t="n">
+      <c r="A465" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="B465" t="inlineStr">
@@ -10131,6 +10131,615 @@
         <v>48</v>
       </c>
       <c r="E465" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C466" t="n">
+        <v>29.06999969482422</v>
+      </c>
+      <c r="D466" t="n">
+        <v>28</v>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C467" t="n">
+        <v>13.30000019073486</v>
+      </c>
+      <c r="D467" t="n">
+        <v>31</v>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C468" t="n">
+        <v>22.71999931335449</v>
+      </c>
+      <c r="D468" t="n">
+        <v>30</v>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C469" t="n">
+        <v>4</v>
+      </c>
+      <c r="D469" t="n">
+        <v>16</v>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C470" t="n">
+        <v>0.7300000190734863</v>
+      </c>
+      <c r="D470" t="n">
+        <v>12</v>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C471" t="n">
+        <v>185.3999938964844</v>
+      </c>
+      <c r="D471" t="n">
+        <v>26</v>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C472" t="n">
+        <v>60.72999954223633</v>
+      </c>
+      <c r="D472" t="n">
+        <v>45</v>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C473" t="n">
+        <v>5.320000171661377</v>
+      </c>
+      <c r="D473" t="n">
+        <v>61</v>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C474" t="n">
+        <v>6.920000076293945</v>
+      </c>
+      <c r="D474" t="n">
+        <v>10</v>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C475" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="D475" t="n">
+        <v>22</v>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C476" t="n">
+        <v>20.29999923706055</v>
+      </c>
+      <c r="D476" t="n">
+        <v>49</v>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C477" t="n">
+        <v>27.65999984741211</v>
+      </c>
+      <c r="D477" t="n">
+        <v>20</v>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C478" t="n">
+        <v>13.14999961853027</v>
+      </c>
+      <c r="D478" t="n">
+        <v>9</v>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C479" t="n">
+        <v>4.800000190734863</v>
+      </c>
+      <c r="D479" t="n">
+        <v>26</v>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C480" t="n">
+        <v>22.94000053405762</v>
+      </c>
+      <c r="D480" t="n">
+        <v>27</v>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C481" t="n">
+        <v>11.97999954223633</v>
+      </c>
+      <c r="D481" t="n">
+        <v>22</v>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C482" t="n">
+        <v>5.920000076293945</v>
+      </c>
+      <c r="D482" t="n">
+        <v>20</v>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C483" t="n">
+        <v>8.109999656677246</v>
+      </c>
+      <c r="D483" t="n">
+        <v>25</v>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C484" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="D484" t="n">
+        <v>30</v>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>49.11999893188477</v>
+      </c>
+      <c r="D485" t="n">
+        <v>23</v>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>4.599999904632568</v>
+      </c>
+      <c r="D486" t="n">
+        <v>20</v>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>64.23999786376953</v>
+      </c>
+      <c r="D487" t="n">
+        <v>8</v>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C488" t="n">
+        <v>51.31999969482422</v>
+      </c>
+      <c r="D488" t="n">
+        <v>16</v>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C489" t="n">
+        <v>19.82999992370605</v>
+      </c>
+      <c r="D489" t="n">
+        <v>63</v>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C490" t="n">
+        <v>38.04999923706055</v>
+      </c>
+      <c r="D490" t="n">
+        <v>35</v>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C491" t="n">
+        <v>112.4700012207031</v>
+      </c>
+      <c r="D491" t="n">
+        <v>31</v>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C492" t="n">
+        <v>48.0099983215332</v>
+      </c>
+      <c r="D492" t="n">
+        <v>11</v>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C493" t="n">
+        <v>7.659999847412109</v>
+      </c>
+      <c r="D493" t="n">
+        <v>11</v>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C494" t="n">
+        <v>38.09000015258789</v>
+      </c>
+      <c r="D494" t="n">
+        <v>48</v>
+      </c>
+      <c r="E494" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>

<commit_message>
chore: atualiza histórico de ordens 2026-09-11
</commit_message>
<xml_diff>
--- a/historico_diario.xlsx
+++ b/historico_diario.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E494"/>
+  <dimension ref="A1:E523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10137,7 +10137,7 @@
       </c>
     </row>
     <row r="466">
-      <c r="A466" s="2" t="n">
+      <c r="A466" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B466" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
     </row>
     <row r="467">
-      <c r="A467" s="2" t="n">
+      <c r="A467" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B467" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
     </row>
     <row r="468">
-      <c r="A468" s="2" t="n">
+      <c r="A468" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B468" t="inlineStr">
@@ -10200,7 +10200,7 @@
       </c>
     </row>
     <row r="469">
-      <c r="A469" s="2" t="n">
+      <c r="A469" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B469" t="inlineStr">
@@ -10221,7 +10221,7 @@
       </c>
     </row>
     <row r="470">
-      <c r="A470" s="2" t="n">
+      <c r="A470" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B470" t="inlineStr">
@@ -10242,7 +10242,7 @@
       </c>
     </row>
     <row r="471">
-      <c r="A471" s="2" t="n">
+      <c r="A471" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B471" t="inlineStr">
@@ -10263,7 +10263,7 @@
       </c>
     </row>
     <row r="472">
-      <c r="A472" s="2" t="n">
+      <c r="A472" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B472" t="inlineStr">
@@ -10284,7 +10284,7 @@
       </c>
     </row>
     <row r="473">
-      <c r="A473" s="2" t="n">
+      <c r="A473" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B473" t="inlineStr">
@@ -10305,7 +10305,7 @@
       </c>
     </row>
     <row r="474">
-      <c r="A474" s="2" t="n">
+      <c r="A474" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B474" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
     </row>
     <row r="475">
-      <c r="A475" s="2" t="n">
+      <c r="A475" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B475" t="inlineStr">
@@ -10347,7 +10347,7 @@
       </c>
     </row>
     <row r="476">
-      <c r="A476" s="2" t="n">
+      <c r="A476" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B476" t="inlineStr">
@@ -10368,7 +10368,7 @@
       </c>
     </row>
     <row r="477">
-      <c r="A477" s="2" t="n">
+      <c r="A477" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B477" t="inlineStr">
@@ -10389,7 +10389,7 @@
       </c>
     </row>
     <row r="478">
-      <c r="A478" s="2" t="n">
+      <c r="A478" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B478" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
     </row>
     <row r="479">
-      <c r="A479" s="2" t="n">
+      <c r="A479" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B479" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
     </row>
     <row r="480">
-      <c r="A480" s="2" t="n">
+      <c r="A480" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B480" t="inlineStr">
@@ -10452,7 +10452,7 @@
       </c>
     </row>
     <row r="481">
-      <c r="A481" s="2" t="n">
+      <c r="A481" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B481" t="inlineStr">
@@ -10473,7 +10473,7 @@
       </c>
     </row>
     <row r="482">
-      <c r="A482" s="2" t="n">
+      <c r="A482" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B482" t="inlineStr">
@@ -10494,7 +10494,7 @@
       </c>
     </row>
     <row r="483">
-      <c r="A483" s="2" t="n">
+      <c r="A483" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B483" t="inlineStr">
@@ -10515,7 +10515,7 @@
       </c>
     </row>
     <row r="484">
-      <c r="A484" s="2" t="n">
+      <c r="A484" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B484" t="inlineStr">
@@ -10536,7 +10536,7 @@
       </c>
     </row>
     <row r="485">
-      <c r="A485" s="2" t="n">
+      <c r="A485" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B485" t="inlineStr">
@@ -10557,7 +10557,7 @@
       </c>
     </row>
     <row r="486">
-      <c r="A486" s="2" t="n">
+      <c r="A486" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B486" t="inlineStr">
@@ -10578,7 +10578,7 @@
       </c>
     </row>
     <row r="487">
-      <c r="A487" s="2" t="n">
+      <c r="A487" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B487" t="inlineStr">
@@ -10599,7 +10599,7 @@
       </c>
     </row>
     <row r="488">
-      <c r="A488" s="2" t="n">
+      <c r="A488" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B488" t="inlineStr">
@@ -10620,7 +10620,7 @@
       </c>
     </row>
     <row r="489">
-      <c r="A489" s="2" t="n">
+      <c r="A489" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B489" t="inlineStr">
@@ -10641,7 +10641,7 @@
       </c>
     </row>
     <row r="490">
-      <c r="A490" s="2" t="n">
+      <c r="A490" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B490" t="inlineStr">
@@ -10662,7 +10662,7 @@
       </c>
     </row>
     <row r="491">
-      <c r="A491" s="2" t="n">
+      <c r="A491" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B491" t="inlineStr">
@@ -10683,7 +10683,7 @@
       </c>
     </row>
     <row r="492">
-      <c r="A492" s="2" t="n">
+      <c r="A492" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B492" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
     </row>
     <row r="493">
-      <c r="A493" s="2" t="n">
+      <c r="A493" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B493" t="inlineStr">
@@ -10725,7 +10725,7 @@
       </c>
     </row>
     <row r="494">
-      <c r="A494" s="2" t="n">
+      <c r="A494" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="B494" t="inlineStr">
@@ -10740,6 +10740,615 @@
         <v>48</v>
       </c>
       <c r="E494" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>ALOS3</t>
+        </is>
+      </c>
+      <c r="C495" t="n">
+        <v>28.63999938964844</v>
+      </c>
+      <c r="D495" t="n">
+        <v>28</v>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="C496" t="n">
+        <v>13.36999988555908</v>
+      </c>
+      <c r="D496" t="n">
+        <v>31</v>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="C497" t="n">
+        <v>22.42000007629395</v>
+      </c>
+      <c r="D497" t="n">
+        <v>30</v>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="C498" t="n">
+        <v>4.130000114440918</v>
+      </c>
+      <c r="D498" t="n">
+        <v>16</v>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>BHIA3</t>
+        </is>
+      </c>
+      <c r="C499" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D499" t="n">
+        <v>12</v>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>BOVA11</t>
+        </is>
+      </c>
+      <c r="C500" t="n">
+        <v>184.2400054931641</v>
+      </c>
+      <c r="D500" t="n">
+        <v>26</v>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="C501" t="n">
+        <v>60.91999816894531</v>
+      </c>
+      <c r="D501" t="n">
+        <v>45</v>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>BRKM5</t>
+        </is>
+      </c>
+      <c r="C502" t="n">
+        <v>5.239999771118164</v>
+      </c>
+      <c r="D502" t="n">
+        <v>61</v>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>CMIN3</t>
+        </is>
+      </c>
+      <c r="C503" t="n">
+        <v>6.690000057220459</v>
+      </c>
+      <c r="D503" t="n">
+        <v>10</v>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="C504" t="n">
+        <v>6.690000057220459</v>
+      </c>
+      <c r="D504" t="n">
+        <v>22</v>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>CXSE3</t>
+        </is>
+      </c>
+      <c r="C505" t="n">
+        <v>19.79000091552734</v>
+      </c>
+      <c r="D505" t="n">
+        <v>49</v>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>ENEV3</t>
+        </is>
+      </c>
+      <c r="C506" t="n">
+        <v>27.40999984741211</v>
+      </c>
+      <c r="D506" t="n">
+        <v>20</v>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>EZTC3</t>
+        </is>
+      </c>
+      <c r="C507" t="n">
+        <v>13.14999961853027</v>
+      </c>
+      <c r="D507" t="n">
+        <v>9</v>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>GMAT3</t>
+        </is>
+      </c>
+      <c r="C508" t="n">
+        <v>4.889999866485596</v>
+      </c>
+      <c r="D508" t="n">
+        <v>26</v>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>HYPE3</t>
+        </is>
+      </c>
+      <c r="C509" t="n">
+        <v>22.78000068664551</v>
+      </c>
+      <c r="D509" t="n">
+        <v>27</v>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>JHSF3</t>
+        </is>
+      </c>
+      <c r="C510" t="n">
+        <v>12.09000015258789</v>
+      </c>
+      <c r="D510" t="n">
+        <v>22</v>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="C511" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="D511" t="n">
+        <v>20</v>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>MOVI3</t>
+        </is>
+      </c>
+      <c r="C512" t="n">
+        <v>7.940000057220459</v>
+      </c>
+      <c r="D512" t="n">
+        <v>25</v>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>MRVE3</t>
+        </is>
+      </c>
+      <c r="C513" t="n">
+        <v>5.769999980926514</v>
+      </c>
+      <c r="D513" t="n">
+        <v>30</v>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="C514" t="n">
+        <v>48.95000076293945</v>
+      </c>
+      <c r="D514" t="n">
+        <v>23</v>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>POMO4</t>
+        </is>
+      </c>
+      <c r="C515" t="n">
+        <v>4.519999980926514</v>
+      </c>
+      <c r="D515" t="n">
+        <v>20</v>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>PRIO3</t>
+        </is>
+      </c>
+      <c r="C516" t="n">
+        <v>63.95000076293945</v>
+      </c>
+      <c r="D516" t="n">
+        <v>8</v>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>PSSA3</t>
+        </is>
+      </c>
+      <c r="C517" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="D517" t="n">
+        <v>16</v>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>RADL3</t>
+        </is>
+      </c>
+      <c r="C518" t="n">
+        <v>19.38999938964844</v>
+      </c>
+      <c r="D518" t="n">
+        <v>63</v>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>RDOR3</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>37.54999923706055</v>
+      </c>
+      <c r="D519" t="n">
+        <v>35</v>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>SMAL11</t>
+        </is>
+      </c>
+      <c r="C520" t="n">
+        <v>110.9700012207031</v>
+      </c>
+      <c r="D520" t="n">
+        <v>31</v>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>SUZB3</t>
+        </is>
+      </c>
+      <c r="C521" t="n">
+        <v>47.97999954223633</v>
+      </c>
+      <c r="D521" t="n">
+        <v>11</v>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>USIM5</t>
+        </is>
+      </c>
+      <c r="C522" t="n">
+        <v>7.360000133514404</v>
+      </c>
+      <c r="D522" t="n">
+        <v>11</v>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>VBBR3</t>
+        </is>
+      </c>
+      <c r="C523" t="n">
+        <v>37.54999923706055</v>
+      </c>
+      <c r="D523" t="n">
+        <v>48</v>
+      </c>
+      <c r="E523" t="inlineStr">
         <is>
           <t>Compra</t>
         </is>

</xml_diff>